<commit_message>
feat(balance): Redesign defense, heal, and buff cards into attack-focused TD tower mechanics
</commit_message>
<xml_diff>
--- a/word_assets_all.xlsx
+++ b/word_assets_all.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1255,12 +1255,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>불</t>
+          <t>방</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>불 (원소/화염)</t>
+          <t>방 (방어/충격파)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1275,35 +1275,35 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="F20" t="n">
         <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>적에게 7 화염 피해를 입히고 3턴간 화상(매 턴 4 피해)을 부여합니다.</t>
+          <t>접근하는 적들에게 12의 방어 충격파를 발사하여 뒤로 밀어내고(넉백) 40% 감속시킵니다.</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/fire_불/fire_1_32px_pastel.png</t>
+          <t>res://assets/02_방어_장비/shield_방/shield_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>물</t>
+          <t>갑</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>물 (원소/수류)</t>
+          <t>갑 (철갑/가시파편)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1318,35 +1318,35 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="F21" t="n">
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>적에게 6 피해를 입히고, 6 방어도를 얻으며 자신의 모든 디버프를 정화합니다.</t>
+          <t>가시 철갑 파편을 사방으로 발사하여 15의 날카로운 관통 물리 피해를 입힙니다.</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/water_물/water_1_32px.png</t>
+          <t>res://assets/02_방어_장비/armor_갑/armor_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>빙</t>
+          <t>문</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>빙 (원소/빙결)</t>
+          <t>문 (관문/철문낙하)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1361,35 +1361,35 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="F22" t="n">
         <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>적을 얼려 7 냉기 피해를 입히고 1턴간 적의 공격력을 4 감소시킵니다.</t>
+          <t>적의 경로 위에 거대한 철문을 쿵 내리찍어 14 피해를 주고 1.5초간 기절(Stun)시킵니다.</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/ice_빙/ice_1_32px_pastel.png</t>
+          <t>res://assets/02_방어_장비/gate_문/gate_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>광</t>
+          <t>성</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>광 (원소/섬광)</t>
+          <t>성 (성채/요새포)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1404,35 +1404,35 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="F23" t="n">
         <v>1</v>
       </c>
       <c r="G23" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>눈부신 섬광을 터뜨려 8 피해를 입히고 적의 이번 턴 공격 의도를 취소시킵니다.</t>
+          <t>요새의 육중한 성채 방어포를 발사하여 18의 광역 포격 피해를 입힙니다.</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/flash_광/flash_1_32px_pastel.png</t>
+          <t>res://assets/02_방어_장비/castle_성/castle_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>노</t>
+          <t>불</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>노 (원소/노을)</t>
+          <t>불 (원소/화염)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1454,28 +1454,28 @@
         <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>타오르는 노을빛으로 8 광역 피해를 입히고 2턴간 화상(매 턴 3)을 부여합니다.</t>
+          <t>적에게 7 화염 피해를 입히고 3턴간 화상(매 턴 4 피해)을 부여합니다.</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/ember_노/ember_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/fire_불/fire_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>암</t>
+          <t>물</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>암 (원소/암흑)</t>
+          <t>물 (원소/수류)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1497,28 +1497,28 @@
         <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>어둠의 파동을 뿜어 9 암흑 피해를 입히고 적 공격력을 2 영구 흡수합니다.</t>
+          <t>적에게 6 피해를 입히고, 6 방어도를 얻으며 자신의 모든 디버프를 정화합니다.</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/darkness_암/darkness_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/water_물/water_1_32px.png</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>우</t>
+          <t>빙</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>우 (원소/뇌우)</t>
+          <t>빙 (원소/빙결)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1540,28 +1540,28 @@
         <v>1</v>
       </c>
       <c r="G26" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>천둥과 폭우를 소환하여 11 뇌전 피해를 입히고 1턴간 적을 실명시킵니다.</t>
+          <t>적을 얼려 7 냉기 피해를 입히고 1턴간 적의 공격력을 4 감소시킵니다.</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/thunder_rain_우/thunder_rain_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/ice_빙/ice_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>와</t>
+          <t>광</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>와 (원소/와류)</t>
+          <t>광 (원소/섬광)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1587,24 +1587,24 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>소용돌이를 일으켜 8 수류 피해를 입히고 적의 방어도를 절반으로 깎습니다.</t>
+          <t>눈부신 섬광을 터뜨려 8 피해를 입히고 적의 이번 턴 공격 의도를 취소시킵니다.</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/whirlpool_water_와/whirlpool_water_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/flash_광/flash_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>얼</t>
+          <t>노</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>얼 (원소/빙하)</t>
+          <t>노 (원소/노을)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1630,24 +1630,24 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>빙하 파편을 꽂아 8 냉기 피해를 입히고 1턴간 적의 공격력을 4 깎습니다.</t>
+          <t>타오르는 노을빛으로 8 광역 피해를 입히고 2턴간 화상(매 턴 3)을 부여합니다.</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/freeze_얼/freeze_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/ember_노/ember_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>업</t>
+          <t>암</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>업 (원소/업화)</t>
+          <t>암 (원소/암흑)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1669,28 +1669,28 @@
         <v>1</v>
       </c>
       <c r="G29" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>인과의 불꽃으로 10 피해를 입히고, 적이 공격할 때마다 4 화염 반사 피해를 줍니다.</t>
+          <t>어둠의 파동을 뿜어 9 암흑 피해를 입히고 적 공격력을 2 영구 흡수합니다.</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/karma_ember_업/karma_ember_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/darkness_암/darkness_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>음</t>
+          <t>우</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>음 (음파/충격)</t>
+          <t>우 (원소/뇌우)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1705,35 +1705,35 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>basic</t>
+          <t>element</t>
         </is>
       </c>
       <c r="F30" t="n">
         <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>강력한 진동 음파로 6 관통 피해를 입히고 적의 마법 시전을 차단합니다.</t>
+          <t>천둥과 폭우를 소환하여 11 뇌전 피해를 입히고 1턴간 적을 실명시킵니다.</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/soundwave_음/soundwave_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/thunder_rain_우/thunder_rain_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>석</t>
+          <t>와</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>석 (자연/투석)</t>
+          <t>와 (원소/와류)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1748,35 +1748,35 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>basic</t>
+          <t>element</t>
         </is>
       </c>
       <c r="F31" t="n">
         <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>단단한 암석을 투척하여 9 물리 피해를 입히고 적 방어도를 5 파괴합니다.</t>
+          <t>소용돌이를 일으켜 8 수류 피해를 입히고 적의 방어도를 절반으로 깎습니다.</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/rock_stone_석/rock_stone_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/whirlpool_water_와/whirlpool_water_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>선</t>
+          <t>얼</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>선 (자연/돌풍)</t>
+          <t>얼 (원소/빙하)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1791,35 +1791,35 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>basic</t>
+          <t>element</t>
         </is>
       </c>
       <c r="F32" t="n">
         <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>돌풍을 소환하여 7 피해를 입히고 날아오는 적 투사체를 튕겨냅니다 (방어도 6).</t>
+          <t>빙하 파편을 꽂아 8 냉기 피해를 입히고 1턴간 적의 공격력을 4 깎습니다.</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/wind_mist_선/wind_mist_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/freeze_얼/freeze_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>수</t>
+          <t>업</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>수 (원소/격류)</t>
+          <t>업 (원소/업화)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1841,28 +1841,28 @@
         <v>1</v>
       </c>
       <c r="G33" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>수류를 방출하여 적에게 8 피해를 입히고 아군에게 6 방어도를 부여합니다.</t>
+          <t>인과의 불꽃으로 10 피해를 입히고, 적이 공격할 때마다 4 화염 반사 피해를 줍니다.</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/water_flow_수/water_flow_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/karma_ember_업/karma_ember_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>뇌</t>
+          <t>음</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>뇌 (원소/뇌전)</t>
+          <t>음 (음파/충격)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1877,35 +1877,35 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>basic</t>
         </is>
       </c>
       <c r="F34" t="n">
         <v>1</v>
       </c>
       <c r="G34" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>천둥 번개를 소환하여 적에게 14의 폭발적인 뇌전 피해를 입힙니다.</t>
+          <t>강력한 진동 음파로 6 관통 피해를 입히고 적의 마법 시전을 차단합니다.</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/lightning_bolt_뇌/lightning_bolt_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/soundwave_음/soundwave_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>곰</t>
+          <t>석</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>곰 (생물/도발)</t>
+          <t>석 (자연/투석)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1920,35 +1920,35 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>summon</t>
+          <t>basic</t>
         </is>
       </c>
       <c r="F35" t="n">
         <v>1</v>
       </c>
       <c r="G35" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>거대한 곰을 소환하여 6 피해를 입히고 8 실드 및 1턴간 도발(피해 흡수)을 겁니다.</t>
+          <t>단단한 암석을 투척하여 9 물리 피해를 입히고 적 방어도를 5 파괴합니다.</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/bear_곰/bear_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/rock_stone_석/rock_stone_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>뱀</t>
+          <t>선</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>뱀 (생물/맹독)</t>
+          <t>선 (자연/돌풍)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1963,35 +1963,35 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>summon</t>
+          <t>basic</t>
         </is>
       </c>
       <c r="F36" t="n">
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>초록 독사를 소환해 4 피해를 입히고 4의 맹독(지속 피해)을 주입합니다.</t>
+          <t>돌풍을 소환하여 7 피해를 입히고 날아오는 적 투사체를 튕겨냅니다 (방어도 6).</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/snake_뱀/snake_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/wind_mist_선/wind_mist_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>말</t>
+          <t>수</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>말 (생물/질주)</t>
+          <t>수 (원소/격류)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>summon</t>
+          <t>element</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -2017,24 +2017,24 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>야생마가 돌진하여 적에게 8 피해를 입히고 이번 턴 즉시 추가 1회 행동을 얻습니다.</t>
+          <t>수류를 방출하여 적에게 8 피해를 입히고 아군에게 6 방어도를 부여합니다.</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/horse_말/horse_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/water_flow_수/water_flow_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>소</t>
+          <t>뇌</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>소 (생물/돌파)</t>
+          <t>뇌 (원소/뇌전)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2049,35 +2049,35 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>summon</t>
+          <t>element</t>
         </is>
       </c>
       <c r="F38" t="n">
         <v>1</v>
       </c>
       <c r="G38" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>황소가 들이받아 11 피해를 입히고 적의 모든 방어도를 완전히 파괴합니다.</t>
+          <t>천둥 번개를 소환하여 적에게 14의 폭발적인 뇌전 피해를 입힙니다.</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/bull_소/bull_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/lightning_bolt_뇌/lightning_bolt_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>개</t>
+          <t>곰</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>개 (생물/충견)</t>
+          <t>곰 (생물/도발)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2099,28 +2099,28 @@
         <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>충견을 소환하여 적에게 5 피해를 입히고 피해를 대신 흡수하는 6 실드를 얻습니다.</t>
+          <t>거대한 곰을 소환하여 6 피해를 입히고 8 실드 및 1턴간 도발(피해 흡수)을 겁니다.</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/dog_wolf_개/dog_wolf_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/bear_곰/bear_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>벌</t>
+          <t>뱀</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>벌 (생물/독침)</t>
+          <t>뱀 (생물/맹독)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2142,28 +2142,28 @@
         <v>1</v>
       </c>
       <c r="G40" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>말벌 떼를 풀어 2 피해를 2회(총 4 피해) 입히고 맹독 3스택을 겁니다.</t>
+          <t>초록 독사를 소환해 4 피해를 입히고 4의 맹독(지속 피해)을 주입합니다.</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/wasp_bee_벌/wasp_bee_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/snake_뱀/snake_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>범</t>
+          <t>말</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>범 (생물/호랑이)</t>
+          <t>말 (생물/질주)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2185,28 +2185,28 @@
         <v>1</v>
       </c>
       <c r="G41" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>호랑이의 포효로 적 전체에 13 피해를 입히고 1턴간 공포(피해량 -50%)를 겁니다.</t>
+          <t>야생마가 돌진하여 적에게 8 피해를 입히고 이번 턴 즉시 추가 1회 행동을 얻습니다.</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/tiger_범/tiger_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/horse_말/horse_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>매</t>
+          <t>소</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>매 (생물/저격)</t>
+          <t>소 (생물/돌파)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2228,28 +2228,28 @@
         <v>1</v>
       </c>
       <c r="G42" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>매가 급강하하여 적의 방어도를 완전히 무시하는 9 관통 피해를 입힙니다.</t>
+          <t>황소가 들이받아 11 피해를 입히고 적의 모든 방어도를 완전히 파괴합니다.</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/hawk_eagle_매/hawk_eagle_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/bull_소/bull_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>낭</t>
+          <t>개</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>낭 (생물/늑대)</t>
+          <t>개 (생물/충견)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2271,28 +2271,28 @@
         <v>1</v>
       </c>
       <c r="G43" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>늑대 무리를 불러 7 피해를 입히고 적의 방어도를 4 깎아냅니다.</t>
+          <t>충견을 소환하여 적에게 5 피해를 입히고 피해를 대신 흡수하는 6 실드를 얻습니다.</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/wolf_낭/wolf_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/dog_wolf_개/dog_wolf_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>솔</t>
+          <t>벌</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>솔 (자연/솔방울)</t>
+          <t>벌 (생물/독침)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2307,35 +2307,35 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>basic</t>
+          <t>summon</t>
         </is>
       </c>
       <c r="F44" t="n">
         <v>1</v>
       </c>
       <c r="G44" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>솔방울 폭탄을 던져 10의 범위 폭발 피해를 입힙니다.</t>
+          <t>말벌 떼를 풀어 2 피해를 2회(총 4 피해) 입히고 맹독 3스택을 겁니다.</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/pinecone_솔/pinecone_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/wasp_bee_벌/wasp_bee_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>입</t>
+          <t>범</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>입 (신체/흡혈)</t>
+          <t>범 (생물/호랑이)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2350,35 +2350,35 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>basic</t>
+          <t>summon</t>
         </is>
       </c>
       <c r="F45" t="n">
         <v>1</v>
       </c>
       <c r="G45" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>적에게 4 피해를 입히고 입힌 피해만큼 체력을 그대로 흡수(흡혈)합니다.</t>
+          <t>호랑이의 포효로 적 전체에 13 피해를 입히고 1턴간 공포(피해량 -50%)를 겁니다.</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>res://assets/06_회복_치유/mouth_blood_입/mouth_blood_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/tiger_범/tiger_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>월</t>
+          <t>매</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>월 (신비/월광)</t>
+          <t>매 (생물/저격)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2393,7 +2393,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>basic</t>
+          <t>summon</t>
         </is>
       </c>
       <c r="F46" t="n">
@@ -2404,24 +2404,24 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>초승달 검기로 9 암흑 피해를 입히고 체력 4를 흡혈합니다.</t>
+          <t>매가 급강하하여 적의 방어도를 완전히 무시하는 9 관통 피해를 입힙니다.</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>res://assets/06_회복_치유/moon_light_월/moon_light_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/hawk_eagle_매/hawk_eagle_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>세</t>
+          <t>낭</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>세 (기세/압도)</t>
+          <t>낭 (생물/늑대)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2436,508 +2436,508 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>basic</t>
+          <t>summon</t>
         </is>
       </c>
       <c r="F47" t="n">
         <v>1</v>
       </c>
       <c r="G47" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>도도한 기세로 8 피해를 입히고 다음 내 카드의 공격력을 +4 증가시킵니다.</t>
+          <t>늑대 무리를 불러 7 피해를 입히고 적의 방어도를 4 깎아냅니다.</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>res://assets/07_버프_유틸/power_surge_세/power_surge_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/wolf_낭/wolf_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>불꽃</t>
+          <t>솔</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>불꽃 (원소/폭발)</t>
+          <t>솔 (자연/솔방울)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>basic</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G48" t="n">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 24의 강력한 광역 화염 폭발을 일으키고 적들을 불태웁니다.</t>
+          <t>솔방울 폭탄을 던져 10의 범위 폭발 피해를 입힙니다.</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/fire_불/fire_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/pinecone_솔/pinecone_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>얼음</t>
+          <t>숨</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>얼음 (원소/빙결)</t>
+          <t>숨 (숨결/영기방출)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>heal</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G49" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 18의 냉기 피해를 주고 적의 이동속도를 75% 둔화시킵니다.</t>
+          <t>전방 부채꼴 범위로 16의 거대한 영기 숨결을 뿜어내어 적들을 지속 피해로 태웁니다.</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/ice_빙/ice_1_32px_pastel.png</t>
+          <t>res://assets/05_회복_치유/breath_숨/breath_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>화살</t>
+          <t>생</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>화살 (무기/원거리)</t>
+          <t>생 (생명/영혼흡수)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>weapon</t>
+          <t>heal</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G50" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 초장거리(220px)에서 22의 관통 화살을 빠르게 사격합니다.</t>
+          <t>적에게 14의 영혼 흡수탄을 발사하며, 적 처치 시 기지 HP를 +1 회복합니다.</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/arrow_시/arrow_1_32px_pastel.png</t>
+          <t>res://assets/05_회복_치유/life_생/life_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>검술</t>
+          <t>샘</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>검술 (무기/연타)</t>
+          <t>샘 (치유샘/물기둥)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>weapon</t>
+          <t>heal</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G51" t="n">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 26의 예리한 검기로 적을 빠르게 2회 연속 베어 넘깁니다.</t>
+          <t>바닥에서 솟구치는 거대한 물기둥을 분출하여 12 피해와 함께 적을 0.5초간 공중으로 띄웁니다.</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/sword_검/sword_1_32px_pastel.png</t>
+          <t>res://assets/05_회복_치유/spring_샘/spring_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>방패</t>
+          <t>입</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>방패 (방어/버프)</t>
+          <t>입 (신체/흡혈)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>defense</t>
+          <t>basic</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G52" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 방어 결계를 펼쳐 주변 모든 아군 타워의 공격속도를 +30% 증폭시킵니다.</t>
+          <t>적에게 4 피해를 입히고 입힌 피해만큼 체력을 그대로 흡수(흡혈)합니다.</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>res://assets/02_방어_보호/shield_방/shield_1_32px_pastel.png</t>
+          <t>res://assets/06_회복_치유/mouth_blood_입/mouth_blood_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>성벽</t>
+          <t>월</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>성벽 (방어/요새)</t>
+          <t>월 (신비/월광)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>defense</t>
+          <t>basic</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G53" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 사거리 내 진입한 적들의 이동속도를 50% 영구 감속시킵니다.</t>
+          <t>초승달 검기로 9 암흑 피해를 입히고 체력 4를 흡혈합니다.</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>res://assets/02_방어_보호/wall_성/wall_1_32px_pastel.png</t>
+          <t>res://assets/06_회복_치유/moon_light_월/moon_light_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>벼락</t>
+          <t>북</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>벼락 (원소/감전)</t>
+          <t>북 (전쟁의북/고동)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>skill</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G54" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 30의 강력한 뇌전을 떨어뜨려 최대 3체의 적에게 연쇄 감전 피해를 입힙니다.</t>
+          <t>둥둥 울리는 북소리로 10 음파 피해를 주며, 주변 아군 타워 공격속도를 +40% 가속합니다.</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/lightning_뇌/lightning_1_32px_pastel.png</t>
+          <t>res://assets/06_버프_유틸/drum_북/drum_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>폭풍</t>
+          <t>기</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>폭풍 (원소/소용돌이)</t>
+          <t>기 (기공/관통기공파)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>skill</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G55" t="n">
         <v>20</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 거대한 소용돌이를 소환하여 범위 내 적들을 지속적으로 갈아냅니다.</t>
+          <t>일직선상 모든 적을 관통하는 푸른 기공파를 발사하여 20의 강력한 관통 피해를 입힙니다.</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/wind_풍/wind_1_32px_pastel.png</t>
+          <t>res://assets/06_버프_유틸/ki_기/ki_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>바람</t>
+          <t>속</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>바람 (원소/돌풍)</t>
+          <t>속 (속도/고속연사)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>skill</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G56" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 강한 돌풍을 날려 적을 뒤로 넉백시킵니다.</t>
+          <t>공격 쿨타임이 0.25초로 극도로 빨라 초당 4회 이상의 고속 활자 난사를 퍼붓습니다.</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/wind_풍/wind_1_32px_pastel.png</t>
+          <t>res://assets/06_버프_유틸/speed_속/speed_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>치유</t>
+          <t>능</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>치유 (회복/성역)</t>
+          <t>능 (능력/마력증폭)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>heal</t>
+          <t>skill</t>
         </is>
       </c>
       <c r="F57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G57" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 매 웨이브 클리어 시 플레이어 기지 체력을 +2 추가 회복합니다.</t>
+          <t>적에게 16 마력 광선을 쏘며 마력 표식을 남겨, 대상이 받는 모든 타워 피해를 +30% 증폭시킵니다.</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>res://assets/06_회복_치유/life_sprout_생/life_sprout_1_32px_pastel.png</t>
+          <t>res://assets/06_버프_유틸/mana_능/mana_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>생명</t>
+          <t>세</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>생명 (회복/축복)</t>
+          <t>세 (기세/압도)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>heal</t>
+          <t>basic</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G58" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 기지의 최대 체력을 +5 영구 증가시킵니다.</t>
+          <t>도도한 기세로 8 피해를 입히고 다음 내 카드의 공격력을 +4 증가시킵니다.</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>res://assets/06_회복_치유/life_sprout_생/life_sprout_1_32px_pastel.png</t>
+          <t>res://assets/07_버프_유틸/power_surge_세/power_surge_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>맹독</t>
+          <t>불꽃</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>맹독 (원소/부식)</t>
+          <t>불꽃 (원소/폭발)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2959,28 +2959,28 @@
         <v>2</v>
       </c>
       <c r="G59" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 적에게 초당 8의 치명적인 맹독 부식 피해를 부여합니다.</t>
+          <t>[2글자 상위 타워] 24의 강력한 광역 화염 폭발을 일으키고 적들을 불태웁니다.</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/dark_orb_암/dark_orb_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/fire_불/fire_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>호랑</t>
+          <t>얼음</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>호랑 (생물/맹수)</t>
+          <t>얼음 (원소/빙결)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2995,35 +2995,35 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>summon</t>
+          <t>element</t>
         </is>
       </c>
       <c r="F60" t="n">
         <v>2</v>
       </c>
       <c r="G60" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 28의 맹수 타격으로 적의 방어도를 무시하고 물어뜯습니다.</t>
+          <t>[2글자 상위 타워] 18의 냉기 피해를 주고 적의 이동속도를 75% 둔화시킵니다.</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/bear_곰/bear_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/ice_빙/ice_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>마법</t>
+          <t>화살</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>마법 (마법/비전)</t>
+          <t>화살 (무기/원거리)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3038,35 +3038,35 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>weapon</t>
         </is>
       </c>
       <c r="F61" t="n">
         <v>2</v>
       </c>
       <c r="G61" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 일직선상의 적을 모두 꿰뚫는 관통 비전 탄환을 발사합니다.</t>
+          <t>[2글자 상위 타워] 초장거리(220px)에서 22의 관통 화살을 빠르게 사격합니다.</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/light_holy_광/light_holy_1_32px_pastel.png</t>
+          <t>res://assets/01_무기_공격/arrow_시/arrow_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>보물</t>
+          <t>검술</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>보물 (유틸/황금)</t>
+          <t>검술 (무기/연타)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3081,35 +3081,35 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>weapon</t>
         </is>
       </c>
       <c r="F62" t="n">
         <v>2</v>
       </c>
       <c r="G62" t="n">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 이 타워가 적을 처치하면 2배의 골드를 획득합니다.</t>
+          <t>[2글자 상위 타워] 26의 예리한 검기로 적을 빠르게 2회 연속 베어 넘깁니다.</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>res://assets/07_버프_유틸/gold_coin_금/gold_coin_1_32px_pastel.png</t>
+          <t>res://assets/01_무기_공격/sword_검/sword_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>강철</t>
+          <t>방패</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>강철 (방어/단련)</t>
+          <t>방패 (방어/버프)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3131,28 +3131,28 @@
         <v>2</v>
       </c>
       <c r="G63" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 단단한 강철 파편을 투척하여 적을 분쇄합니다.</t>
+          <t>[2글자 상위 타워] 방어 결계를 펼쳐 주변 모든 아군 타워의 공격속도를 +30% 증폭시킵니다.</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/sword_검/sword_1_32px_pastel.png</t>
+          <t>res://assets/02_방어_보호/shield_방/shield_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>화염</t>
+          <t>성벽</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>화염 (원소/업화)</t>
+          <t>성벽 (방어/요새)</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3167,88 +3167,88 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="F64" t="n">
         <v>2</v>
       </c>
       <c r="G64" t="n">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 전방 부채꼴 범위에 27 피해의 지속 화염 방사를 뿜어냅니다.</t>
+          <t>[2글자 상위 타워] 사거리 내 진입한 적들의 이동속도를 50% 영구 감속시킵니다.</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/fire_불/fire_1_32px_pastel.png</t>
+          <t>res://assets/02_방어_보호/wall_성/wall_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>호랑이</t>
+          <t>벼락</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>호랑이 (생물/신수)</t>
+          <t>벼락 (원소/감전)</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>3글자</t>
+          <t>2글자</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>3티어 (신화)</t>
+          <t>2티어 (상위)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>summon</t>
+          <t>element</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G65" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>[3글자 신화 타워] 50의 압도적인 맹수 포효로 적들을 공포에 질리게 하고 전방을 도륙합니다.</t>
+          <t>[2글자 상위 타워] 30의 강력한 뇌전을 떨어뜨려 최대 3체의 적에게 연쇄 감전 피해를 입힙니다.</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/bear_곰/bear_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/lightning_뇌/lightning_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>불벼락</t>
+          <t>폭풍</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>불벼락 (원소/천벌)</t>
+          <t>폭풍 (원소/소용돌이)</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>3글자</t>
+          <t>2글자</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>3티어 (신화)</t>
+          <t>2티어 (상위)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3257,41 +3257,41 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G66" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>[3글자 신화 타워] 60의 화염 낙뢰 폭격으로 화면 내 다수의 적을 일격에 궤멸시킵니다.</t>
+          <t>[2글자 상위 타워] 거대한 소용돌이를 소환하여 범위 내 적들을 지속적으로 갈아냅니다.</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/fire_불/fire_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/wind_풍/wind_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>폭풍우</t>
+          <t>바람</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>폭풍우 (원소/재앙)</t>
+          <t>바람 (원소/돌풍)</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>3글자</t>
+          <t>2글자</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>3티어 (신화)</t>
+          <t>2티어 (상위)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3300,14 +3300,14 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G67" t="n">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>[3글자 신화 타워] 거대한 비바람 태풍을 일으켜 적 전체를 80% 슬로우 상태로 묶어둡니다.</t>
+          <t>[2글자 상위 타워] 강한 돌풍을 날려 적을 뒤로 넉백시킵니다.</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3319,256 +3319,729 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>얼음검</t>
+          <t>치유</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>얼음검 (무기/동결)</t>
+          <t>치유 (회복/성역)</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>3글자</t>
+          <t>2글자</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>3티어 (신화)</t>
+          <t>2티어 (상위)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>weapon</t>
+          <t>heal</t>
         </is>
       </c>
       <c r="F68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G68" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>[3글자 신화 타워] 42의 절대영도 검기로 적을 베는 즉시 2초간 완전히 얼려 멈춥니다.</t>
+          <t>[2글자 상위 타워] 매 웨이브 클리어 시 플레이어 기지 체력을 +2 추가 회복합니다.</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/sword_검/sword_1_32px_pastel.png</t>
+          <t>res://assets/06_회복_치유/life_sprout_생/life_sprout_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>독화살</t>
+          <t>생명</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>독화살 (무기/맹독)</t>
+          <t>생명 (회복/축복)</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>3글자</t>
+          <t>2글자</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>3티어 (신화)</t>
+          <t>2티어 (상위)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>weapon</t>
+          <t>heal</t>
         </is>
       </c>
       <c r="F69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G69" t="n">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>[3글자 신화 타워] 38 피해와 함께 초당 15의 치사량 맹독을 주입하는 화살을 난사합니다.</t>
+          <t>[2글자 상위 타워] 기지의 최대 체력을 +5 영구 증가시킵니다.</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/arrow_시/arrow_1_32px_pastel.png</t>
+          <t>res://assets/06_회복_치유/life_sprout_생/life_sprout_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>대검술</t>
+          <t>맹독</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>대검술 (무기/오의)</t>
+          <t>맹독 (원소/부식)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>3글자</t>
+          <t>2글자</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>3티어 (신화)</t>
+          <t>2티어 (상위)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>weapon</t>
+          <t>element</t>
         </is>
       </c>
       <c r="F70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G70" t="n">
-        <v>55</v>
+        <v>16</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>[3글자 신화 타워] 55의 초대형 참격 검기를 날려 경로 위의 모든 적을 일도양단합니다.</t>
+          <t>[2글자 상위 타워] 적에게 초당 8의 치명적인 맹독 부식 피해를 부여합니다.</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/sword_검/sword_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/dark_orb_암/dark_orb_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>용의숨</t>
+          <t>호랑</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>용의숨 (원소/신화)</t>
+          <t>호랑 (생물/맹수)</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>3글자</t>
+          <t>2글자</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>3티어 (신화)</t>
+          <t>2티어 (상위)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>summon</t>
         </is>
       </c>
       <c r="F71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G71" t="n">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>[3글자 신화 타워] 70의 신화급 드래곤 브레스를 뿜어 전방의 모든 적을 잿더미로 만듭니다.</t>
+          <t>[2글자 상위 타워] 28의 맹수 타격으로 적의 방어도를 무시하고 물어뜯습니다.</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/dragon_용/dragon_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/bear_곰/bear_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>생명수</t>
+          <t>마법</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>생명수 (회복/기적)</t>
+          <t>마법 (마법/비전)</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>3글자</t>
+          <t>2글자</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>3티어 (신화)</t>
+          <t>2티어 (상위)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>heal</t>
+          <t>element</t>
         </is>
       </c>
       <c r="F72" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G72" t="n">
         <v>25</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>[3글자 신화 타워] 기지 체력을 즉시 +5 회복하고, 전 필드 아군 타워 공속을 +50% 버프합니다.</t>
+          <t>[2글자 상위 타워] 일직선상의 적을 모두 꿰뚫는 관통 비전 탄환을 발사합니다.</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>res://assets/06_회복_치유/life_sprout_생/life_sprout_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/light_holy_광/light_holy_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
+          <t>보물</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>보물 (유틸/황금)</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>2글자</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>2티어 (상위)</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>skill</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>2</v>
+      </c>
+      <c r="G73" t="n">
+        <v>12</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>[2글자 상위 타워] 이 타워가 적을 처치하면 2배의 골드를 획득합니다.</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>res://assets/07_버프_유틸/gold_coin_금/gold_coin_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>강철</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>강철 (방어/단련)</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>2글자</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>2티어 (상위)</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>defense</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>2</v>
+      </c>
+      <c r="G74" t="n">
+        <v>20</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>[2글자 상위 타워] 단단한 강철 파편을 투척하여 적을 분쇄합니다.</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>res://assets/01_무기_공격/sword_검/sword_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>화염</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>화염 (원소/업화)</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>2글자</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>2티어 (상위)</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>2</v>
+      </c>
+      <c r="G75" t="n">
+        <v>27</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>[2글자 상위 타워] 전방 부채꼴 범위에 27 피해의 지속 화염 방사를 뿜어냅니다.</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>res://assets/03_원소_마법/fire_불/fire_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>호랑이</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>호랑이 (생물/신수)</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>3글자</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>3티어 (신화)</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>summon</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>3</v>
+      </c>
+      <c r="G76" t="n">
+        <v>50</v>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>[3글자 신화 타워] 50의 압도적인 맹수 포효로 적들을 공포에 질리게 하고 전방을 도륙합니다.</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>res://assets/04_생물_소환/bear_곰/bear_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>불벼락</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>불벼락 (원소/천벌)</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>3글자</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>3티어 (신화)</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>3</v>
+      </c>
+      <c r="G77" t="n">
+        <v>60</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>[3글자 신화 타워] 60의 화염 낙뢰 폭격으로 화면 내 다수의 적을 일격에 궤멸시킵니다.</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>res://assets/03_원소_마법/fire_불/fire_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>폭풍우</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>폭풍우 (원소/재앙)</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>3글자</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>3티어 (신화)</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>3</v>
+      </c>
+      <c r="G78" t="n">
+        <v>45</v>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>[3글자 신화 타워] 거대한 비바람 태풍을 일으켜 적 전체를 80% 슬로우 상태로 묶어둡니다.</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>res://assets/03_원소_마법/wind_풍/wind_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>얼음검</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>얼음검 (무기/동결)</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>3글자</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>3티어 (신화)</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>3</v>
+      </c>
+      <c r="G79" t="n">
+        <v>42</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>[3글자 신화 타워] 42의 절대영도 검기로 적을 베는 즉시 2초간 완전히 얼려 멈춥니다.</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>res://assets/01_무기_공격/sword_검/sword_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>독화살</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>독화살 (무기/맹독)</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>3글자</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>3티어 (신화)</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>3</v>
+      </c>
+      <c r="G80" t="n">
+        <v>38</v>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>[3글자 신화 타워] 38 피해와 함께 초당 15의 치사량 맹독을 주입하는 화살을 난사합니다.</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>res://assets/01_무기_공격/arrow_시/arrow_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>대검술</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>대검술 (무기/오의)</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>3글자</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>3티어 (신화)</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>3</v>
+      </c>
+      <c r="G81" t="n">
+        <v>55</v>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>[3글자 신화 타워] 55의 초대형 참격 검기를 날려 경로 위의 모든 적을 일도양단합니다.</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>res://assets/01_무기_공격/sword_검/sword_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>용의숨</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>용의숨 (원소/신화)</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>3글자</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>3티어 (신화)</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>3</v>
+      </c>
+      <c r="G82" t="n">
+        <v>70</v>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>[3글자 신화 타워] 70의 신화급 드래곤 브레스를 뿜어 전방의 모든 적을 잿더미로 만듭니다.</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>res://assets/04_생물_소환/dragon_용/dragon_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>생명수</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>생명수 (회복/기적)</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>3글자</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>3티어 (신화)</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>heal</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>3</v>
+      </c>
+      <c r="G83" t="n">
+        <v>25</v>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>[3글자 신화 타워] 기지 체력을 즉시 +5 회복하고, 전 필드 아군 타워 공속을 +50% 버프합니다.</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>res://assets/06_회복_치유/life_sprout_생/life_sprout_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
           <t>철옹성</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B84" t="inlineStr">
         <is>
           <t>철옹성 (방어/무적)</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>3글자</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D84" t="inlineStr">
         <is>
           <t>3티어 (신화)</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
+      <c r="E84" t="inlineStr">
         <is>
           <t>defense</t>
         </is>
       </c>
-      <c r="F73" t="n">
+      <c r="F84" t="n">
         <v>3</v>
       </c>
-      <c r="G73" t="n">
+      <c r="G84" t="n">
         <v>30</v>
       </c>
-      <c r="H73" t="inlineStr">
+      <c r="H84" t="inlineStr">
         <is>
           <t>[3글자 신화 타워] 절대적인 방어 요새를 구축하여 기지에 가해지는 피해를 대폭 흡수합니다.</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr">
+      <c r="I84" t="inlineStr">
         <is>
           <t>res://assets/02_방어_보호/wall_성/wall_1_32px_pastel.png</t>
         </is>

</xml_diff>

<commit_message>
feat(balance): Complete conversion of all defense, heal, and buff words to attack-focused TD towers
</commit_message>
<xml_diff>
--- a/word_assets_all.xlsx
+++ b/word_assets_all.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I84"/>
+  <dimension ref="A1:I96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1427,12 +1427,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>불</t>
+          <t>산</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>불 (원소/화염)</t>
+          <t>산 (태산/낙석)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1447,35 +1447,35 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="F24" t="n">
         <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>적에게 7 화염 피해를 입히고 3턴간 화상(매 턴 4 피해)을 부여합니다.</t>
+          <t>태산 같은 거대한 낙석을 떨어뜨려 18의 광역 물리 피해를 입히고 적들을 크게 밀어냅니다.</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/fire_불/fire_1_32px_pastel.png</t>
+          <t>res://assets/02_방어_장비/mountain_산/mountain_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>물</t>
+          <t>막</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>물 (원소/수류)</t>
+          <t>막 (결계/감속장막)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1490,35 +1490,35 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="F25" t="n">
         <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>적에게 6 피해를 입히고, 6 방어도를 얻으며 자신의 모든 디버프를 정화합니다.</t>
+          <t>지나가는 적에게 12의 마법 장막 충격을 가하며 이동속도를 50% 크게 감속시킵니다.</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/water_물/water_1_32px.png</t>
+          <t>res://assets/02_방어_장비/barrier_막/barrier_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>빙</t>
+          <t>완</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>빙 (원소/빙결)</t>
+          <t>완 (완벽/철퇴타격)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1533,35 +1533,35 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="F26" t="n">
         <v>1</v>
       </c>
       <c r="G26" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>적을 얼려 7 냉기 피해를 입히고 1턴간 적의 공격력을 4 감소시킵니다.</t>
+          <t>완벽한 타이밍의 묵직한 철퇴 강타로 16 단일 물리 피해를 주고 0.8초간 기절시킵니다.</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/ice_빙/ice_1_32px_pastel.png</t>
+          <t>res://assets/02_방어_장비/guard_완/guard_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>광</t>
+          <t>인</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>광 (원소/섬광)</t>
+          <t>인 (인내/강철탄)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1576,35 +1576,35 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="F27" t="n">
         <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>눈부신 섬광을 터뜨려 8 피해를 입히고 적의 이번 턴 공격 의도를 취소시킵니다.</t>
+          <t>강철 같은 단단한 탄환을 쏘아보내어 14의 묵직한 단일 관통 피해를 입힙니다.</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/flash_광/flash_1_32px_pastel.png</t>
+          <t>res://assets/02_방어_장비/patience_인/patience_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>노</t>
+          <t>언</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>노 (원소/노을)</t>
+          <t>언 (언약/신성광선)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1619,35 +1619,35 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="F28" t="n">
         <v>1</v>
       </c>
       <c r="G28" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>타오르는 노을빛으로 8 광역 피해를 입히고 2턴간 화상(매 턴 3)을 부여합니다.</t>
+          <t>신성의 언약 빛기둥을 내리꽂아 15의 신성 광역 피해를 적들에게 가합니다.</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/ember_노/ember_1_32px_pastel.png</t>
+          <t>res://assets/02_방어_장비/pledge_언/pledge_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>암</t>
+          <t>위</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>암 (원소/암흑)</t>
+          <t>위 (위성/궤도레이저)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1662,35 +1662,35 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="F29" t="n">
         <v>1</v>
       </c>
       <c r="G29" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>어둠의 파동을 뿜어 9 암흑 피해를 입히고 적 공격력을 2 영구 흡수합니다.</t>
+          <t>주변을 회전하는 궤도 레이저를 연사하여 13의 지속 마법 피해를 입힙니다.</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/darkness_암/darkness_1_32px_pastel.png</t>
+          <t>res://assets/02_방어_장비/orbit_위/orbit_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>우</t>
+          <t>불</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>우 (원소/뇌우)</t>
+          <t>불 (원소/화염)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1712,28 +1712,28 @@
         <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>천둥과 폭우를 소환하여 11 뇌전 피해를 입히고 1턴간 적을 실명시킵니다.</t>
+          <t>적에게 7 화염 피해를 입히고 3턴간 화상(매 턴 4 피해)을 부여합니다.</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/thunder_rain_우/thunder_rain_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/fire_불/fire_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>와</t>
+          <t>물</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>와 (원소/와류)</t>
+          <t>물 (원소/수류)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1755,28 +1755,28 @@
         <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>소용돌이를 일으켜 8 수류 피해를 입히고 적의 방어도를 절반으로 깎습니다.</t>
+          <t>적에게 6 피해를 입히고, 6 방어도를 얻으며 자신의 모든 디버프를 정화합니다.</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/whirlpool_water_와/whirlpool_water_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/water_물/water_1_32px.png</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>얼</t>
+          <t>빙</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>얼 (원소/빙하)</t>
+          <t>빙 (원소/빙결)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1798,28 +1798,28 @@
         <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>빙하 파편을 꽂아 8 냉기 피해를 입히고 1턴간 적의 공격력을 4 깎습니다.</t>
+          <t>적을 얼려 7 냉기 피해를 입히고 1턴간 적의 공격력을 4 감소시킵니다.</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/freeze_얼/freeze_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/ice_빙/ice_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>업</t>
+          <t>광</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>업 (원소/업화)</t>
+          <t>광 (원소/섬광)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1841,28 +1841,28 @@
         <v>1</v>
       </c>
       <c r="G33" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>인과의 불꽃으로 10 피해를 입히고, 적이 공격할 때마다 4 화염 반사 피해를 줍니다.</t>
+          <t>눈부신 섬광을 터뜨려 8 피해를 입히고 적의 이번 턴 공격 의도를 취소시킵니다.</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/karma_ember_업/karma_ember_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/flash_광/flash_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>음</t>
+          <t>노</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>음 (음파/충격)</t>
+          <t>노 (원소/노을)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1877,35 +1877,35 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>basic</t>
+          <t>element</t>
         </is>
       </c>
       <c r="F34" t="n">
         <v>1</v>
       </c>
       <c r="G34" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>강력한 진동 음파로 6 관통 피해를 입히고 적의 마법 시전을 차단합니다.</t>
+          <t>타오르는 노을빛으로 8 광역 피해를 입히고 2턴간 화상(매 턴 3)을 부여합니다.</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/soundwave_음/soundwave_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/ember_노/ember_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>석</t>
+          <t>암</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>석 (자연/투석)</t>
+          <t>암 (원소/암흑)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>basic</t>
+          <t>element</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -1931,24 +1931,24 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>단단한 암석을 투척하여 9 물리 피해를 입히고 적 방어도를 5 파괴합니다.</t>
+          <t>어둠의 파동을 뿜어 9 암흑 피해를 입히고 적 공격력을 2 영구 흡수합니다.</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/rock_stone_석/rock_stone_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/darkness_암/darkness_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>선</t>
+          <t>우</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>선 (자연/돌풍)</t>
+          <t>우 (원소/뇌우)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1963,35 +1963,35 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>basic</t>
+          <t>element</t>
         </is>
       </c>
       <c r="F36" t="n">
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>돌풍을 소환하여 7 피해를 입히고 날아오는 적 투사체를 튕겨냅니다 (방어도 6).</t>
+          <t>천둥과 폭우를 소환하여 11 뇌전 피해를 입히고 1턴간 적을 실명시킵니다.</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/wind_mist_선/wind_mist_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/thunder_rain_우/thunder_rain_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>수</t>
+          <t>와</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>수 (원소/격류)</t>
+          <t>와 (원소/와류)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2017,24 +2017,24 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>수류를 방출하여 적에게 8 피해를 입히고 아군에게 6 방어도를 부여합니다.</t>
+          <t>소용돌이를 일으켜 8 수류 피해를 입히고 적의 방어도를 절반으로 깎습니다.</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/water_flow_수/water_flow_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/whirlpool_water_와/whirlpool_water_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>뇌</t>
+          <t>얼</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>뇌 (원소/뇌전)</t>
+          <t>얼 (원소/빙하)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2056,28 +2056,28 @@
         <v>1</v>
       </c>
       <c r="G38" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>천둥 번개를 소환하여 적에게 14의 폭발적인 뇌전 피해를 입힙니다.</t>
+          <t>빙하 파편을 꽂아 8 냉기 피해를 입히고 1턴간 적의 공격력을 4 깎습니다.</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/lightning_bolt_뇌/lightning_bolt_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/freeze_얼/freeze_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>곰</t>
+          <t>업</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>곰 (생물/도발)</t>
+          <t>업 (원소/업화)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2092,35 +2092,35 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>summon</t>
+          <t>element</t>
         </is>
       </c>
       <c r="F39" t="n">
         <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>거대한 곰을 소환하여 6 피해를 입히고 8 실드 및 1턴간 도발(피해 흡수)을 겁니다.</t>
+          <t>인과의 불꽃으로 10 피해를 입히고, 적이 공격할 때마다 4 화염 반사 피해를 줍니다.</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/bear_곰/bear_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/karma_ember_업/karma_ember_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>뱀</t>
+          <t>음</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>뱀 (생물/맹독)</t>
+          <t>음 (음파/충격)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2135,35 +2135,35 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>summon</t>
+          <t>basic</t>
         </is>
       </c>
       <c r="F40" t="n">
         <v>1</v>
       </c>
       <c r="G40" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>초록 독사를 소환해 4 피해를 입히고 4의 맹독(지속 피해)을 주입합니다.</t>
+          <t>강력한 진동 음파로 6 관통 피해를 입히고 적의 마법 시전을 차단합니다.</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/snake_뱀/snake_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/soundwave_음/soundwave_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>말</t>
+          <t>석</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>말 (생물/질주)</t>
+          <t>석 (자연/투석)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2178,35 +2178,35 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>summon</t>
+          <t>basic</t>
         </is>
       </c>
       <c r="F41" t="n">
         <v>1</v>
       </c>
       <c r="G41" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>야생마가 돌진하여 적에게 8 피해를 입히고 이번 턴 즉시 추가 1회 행동을 얻습니다.</t>
+          <t>단단한 암석을 투척하여 9 물리 피해를 입히고 적 방어도를 5 파괴합니다.</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/horse_말/horse_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/rock_stone_석/rock_stone_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>소</t>
+          <t>선</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>소 (생물/돌파)</t>
+          <t>선 (자연/돌풍)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2221,35 +2221,35 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>summon</t>
+          <t>basic</t>
         </is>
       </c>
       <c r="F42" t="n">
         <v>1</v>
       </c>
       <c r="G42" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>황소가 들이받아 11 피해를 입히고 적의 모든 방어도를 완전히 파괴합니다.</t>
+          <t>돌풍을 소환하여 7 피해를 입히고 날아오는 적 투사체를 튕겨냅니다 (방어도 6).</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/bull_소/bull_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/wind_mist_선/wind_mist_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>개</t>
+          <t>수</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>개 (생물/충견)</t>
+          <t>수 (원소/격류)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2264,35 +2264,35 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>summon</t>
+          <t>element</t>
         </is>
       </c>
       <c r="F43" t="n">
         <v>1</v>
       </c>
       <c r="G43" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>충견을 소환하여 적에게 5 피해를 입히고 피해를 대신 흡수하는 6 실드를 얻습니다.</t>
+          <t>수류를 방출하여 적에게 8 피해를 입히고 아군에게 6 방어도를 부여합니다.</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/dog_wolf_개/dog_wolf_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/water_flow_수/water_flow_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>벌</t>
+          <t>뇌</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>벌 (생물/독침)</t>
+          <t>뇌 (원소/뇌전)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2307,35 +2307,35 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>summon</t>
+          <t>element</t>
         </is>
       </c>
       <c r="F44" t="n">
         <v>1</v>
       </c>
       <c r="G44" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>말벌 떼를 풀어 2 피해를 2회(총 4 피해) 입히고 맹독 3스택을 겁니다.</t>
+          <t>천둥 번개를 소환하여 적에게 14의 폭발적인 뇌전 피해를 입힙니다.</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/wasp_bee_벌/wasp_bee_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/lightning_bolt_뇌/lightning_bolt_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>범</t>
+          <t>곰</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>범 (생물/호랑이)</t>
+          <t>곰 (생물/도발)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2357,28 +2357,28 @@
         <v>1</v>
       </c>
       <c r="G45" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>호랑이의 포효로 적 전체에 13 피해를 입히고 1턴간 공포(피해량 -50%)를 겁니다.</t>
+          <t>거대한 곰을 소환하여 6 피해를 입히고 8 실드 및 1턴간 도발(피해 흡수)을 겁니다.</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/tiger_범/tiger_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/bear_곰/bear_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>매</t>
+          <t>뱀</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>매 (생물/저격)</t>
+          <t>뱀 (생물/맹독)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2400,28 +2400,28 @@
         <v>1</v>
       </c>
       <c r="G46" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>매가 급강하하여 적의 방어도를 완전히 무시하는 9 관통 피해를 입힙니다.</t>
+          <t>초록 독사를 소환해 4 피해를 입히고 4의 맹독(지속 피해)을 주입합니다.</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/hawk_eagle_매/hawk_eagle_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/snake_뱀/snake_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>낭</t>
+          <t>말</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>낭 (생물/늑대)</t>
+          <t>말 (생물/질주)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2443,28 +2443,28 @@
         <v>1</v>
       </c>
       <c r="G47" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>늑대 무리를 불러 7 피해를 입히고 적의 방어도를 4 깎아냅니다.</t>
+          <t>야생마가 돌진하여 적에게 8 피해를 입히고 이번 턴 즉시 추가 1회 행동을 얻습니다.</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/wolf_낭/wolf_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/horse_말/horse_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>솔</t>
+          <t>소</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>솔 (자연/솔방울)</t>
+          <t>소 (생물/돌파)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2479,35 +2479,35 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>basic</t>
+          <t>summon</t>
         </is>
       </c>
       <c r="F48" t="n">
         <v>1</v>
       </c>
       <c r="G48" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>솔방울 폭탄을 던져 10의 범위 폭발 피해를 입힙니다.</t>
+          <t>황소가 들이받아 11 피해를 입히고 적의 모든 방어도를 완전히 파괴합니다.</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/pinecone_솔/pinecone_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/bull_소/bull_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>숨</t>
+          <t>개</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>숨 (숨결/영기방출)</t>
+          <t>개 (생물/충견)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2522,35 +2522,35 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>heal</t>
+          <t>summon</t>
         </is>
       </c>
       <c r="F49" t="n">
         <v>1</v>
       </c>
       <c r="G49" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>전방 부채꼴 범위로 16의 거대한 영기 숨결을 뿜어내어 적들을 지속 피해로 태웁니다.</t>
+          <t>충견을 소환하여 적에게 5 피해를 입히고 피해를 대신 흡수하는 6 실드를 얻습니다.</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>res://assets/05_회복_치유/breath_숨/breath_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/dog_wolf_개/dog_wolf_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>생</t>
+          <t>벌</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>생 (생명/영혼흡수)</t>
+          <t>벌 (생물/독침)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2565,35 +2565,35 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>heal</t>
+          <t>summon</t>
         </is>
       </c>
       <c r="F50" t="n">
         <v>1</v>
       </c>
       <c r="G50" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>적에게 14의 영혼 흡수탄을 발사하며, 적 처치 시 기지 HP를 +1 회복합니다.</t>
+          <t>말벌 떼를 풀어 2 피해를 2회(총 4 피해) 입히고 맹독 3스택을 겁니다.</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>res://assets/05_회복_치유/life_생/life_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/wasp_bee_벌/wasp_bee_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>샘</t>
+          <t>범</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>샘 (치유샘/물기둥)</t>
+          <t>범 (생물/호랑이)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2608,35 +2608,35 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>heal</t>
+          <t>summon</t>
         </is>
       </c>
       <c r="F51" t="n">
         <v>1</v>
       </c>
       <c r="G51" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>바닥에서 솟구치는 거대한 물기둥을 분출하여 12 피해와 함께 적을 0.5초간 공중으로 띄웁니다.</t>
+          <t>호랑이의 포효로 적 전체에 13 피해를 입히고 1턴간 공포(피해량 -50%)를 겁니다.</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>res://assets/05_회복_치유/spring_샘/spring_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/tiger_범/tiger_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>입</t>
+          <t>매</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>입 (신체/흡혈)</t>
+          <t>매 (생물/저격)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2651,35 +2651,35 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>basic</t>
+          <t>summon</t>
         </is>
       </c>
       <c r="F52" t="n">
         <v>1</v>
       </c>
       <c r="G52" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>적에게 4 피해를 입히고 입힌 피해만큼 체력을 그대로 흡수(흡혈)합니다.</t>
+          <t>매가 급강하하여 적의 방어도를 완전히 무시하는 9 관통 피해를 입힙니다.</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>res://assets/06_회복_치유/mouth_blood_입/mouth_blood_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/hawk_eagle_매/hawk_eagle_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>월</t>
+          <t>낭</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>월 (신비/월광)</t>
+          <t>낭 (생물/늑대)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2694,35 +2694,35 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>basic</t>
+          <t>summon</t>
         </is>
       </c>
       <c r="F53" t="n">
         <v>1</v>
       </c>
       <c r="G53" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>초승달 검기로 9 암흑 피해를 입히고 체력 4를 흡혈합니다.</t>
+          <t>늑대 무리를 불러 7 피해를 입히고 적의 방어도를 4 깎아냅니다.</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>res://assets/06_회복_치유/moon_light_월/moon_light_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/wolf_낭/wolf_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>북</t>
+          <t>솔</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>북 (전쟁의북/고동)</t>
+          <t>솔 (자연/솔방울)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>basic</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -2748,24 +2748,24 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>둥둥 울리는 북소리로 10 음파 피해를 주며, 주변 아군 타워 공격속도를 +40% 가속합니다.</t>
+          <t>솔방울 폭탄을 던져 10의 범위 폭발 피해를 입힙니다.</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>res://assets/06_버프_유틸/drum_북/drum_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/pinecone_솔/pinecone_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>기</t>
+          <t>숨</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>기 (기공/관통기공파)</t>
+          <t>숨 (숨결/영기방출)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2780,35 +2780,35 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>heal</t>
         </is>
       </c>
       <c r="F55" t="n">
         <v>1</v>
       </c>
       <c r="G55" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>일직선상 모든 적을 관통하는 푸른 기공파를 발사하여 20의 강력한 관통 피해를 입힙니다.</t>
+          <t>전방 부채꼴 범위로 16의 거대한 영기 숨결을 뿜어내어 적들을 지속 피해로 태웁니다.</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>res://assets/06_버프_유틸/ki_기/ki_1_32px_pastel.png</t>
+          <t>res://assets/05_회복_치유/breath_숨/breath_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>속</t>
+          <t>생</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>속 (속도/고속연사)</t>
+          <t>생 (생명/영혼흡수)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2823,35 +2823,35 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>heal</t>
         </is>
       </c>
       <c r="F56" t="n">
         <v>1</v>
       </c>
       <c r="G56" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>공격 쿨타임이 0.25초로 극도로 빨라 초당 4회 이상의 고속 활자 난사를 퍼붓습니다.</t>
+          <t>적에게 14의 영혼 흡수탄을 발사하며, 적 처치 시 기지 HP를 +1 회복합니다.</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>res://assets/06_버프_유틸/speed_속/speed_1_32px_pastel.png</t>
+          <t>res://assets/05_회복_치유/life_생/life_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>능</t>
+          <t>샘</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>능 (능력/마력증폭)</t>
+          <t>샘 (치유샘/물기둥)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2866,35 +2866,35 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>heal</t>
         </is>
       </c>
       <c r="F57" t="n">
         <v>1</v>
       </c>
       <c r="G57" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>적에게 16 마력 광선을 쏘며 마력 표식을 남겨, 대상이 받는 모든 타워 피해를 +30% 증폭시킵니다.</t>
+          <t>바닥에서 솟구치는 거대한 물기둥을 분출하여 12 피해와 함께 적을 0.5초간 공중으로 띄웁니다.</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>res://assets/06_버프_유틸/mana_능/mana_1_32px_pastel.png</t>
+          <t>res://assets/05_회복_치유/spring_샘/spring_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>세</t>
+          <t>감</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>세 (기세/압도)</t>
+          <t>감 (단감/투척)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2909,551 +2909,551 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>basic</t>
+          <t>heal</t>
         </is>
       </c>
       <c r="F58" t="n">
         <v>1</v>
       </c>
       <c r="G58" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>도도한 기세로 8 피해를 입히고 다음 내 카드의 공격력을 +4 증가시킵니다.</t>
+          <t>단단한 감 열매를 고속 투척하여 11 피해를 입히고 적을 30% 둔화시킵니다.</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>res://assets/07_버프_유틸/power_surge_세/power_surge_1_32px_pastel.png</t>
+          <t>res://assets/05_회복_치유/persimmon_감/persimmon_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>불꽃</t>
+          <t>식</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>불꽃 (원소/폭발)</t>
+          <t>식 (보양/독초폭탄)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>heal</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G59" t="n">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 24의 강력한 광역 화염 폭발을 일으키고 적들을 불태웁니다.</t>
+          <t>폭발하는 독초 주머니를 던져 13 광역 피해를 입히고 초당 4의 중독 피해를 남깁니다.</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/fire_불/fire_1_32px_pastel.png</t>
+          <t>res://assets/05_회복_치유/food_식/food_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>얼음</t>
+          <t>입</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>얼음 (원소/빙결)</t>
+          <t>입 (신체/흡혈)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>basic</t>
         </is>
       </c>
       <c r="F60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G60" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 18의 냉기 피해를 주고 적의 이동속도를 75% 둔화시킵니다.</t>
+          <t>적에게 4 피해를 입히고 입힌 피해만큼 체력을 그대로 흡수(흡혈)합니다.</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/ice_빙/ice_1_32px_pastel.png</t>
+          <t>res://assets/06_회복_치유/mouth_blood_입/mouth_blood_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>화살</t>
+          <t>월</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>화살 (무기/원거리)</t>
+          <t>월 (신비/월광)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>weapon</t>
+          <t>basic</t>
         </is>
       </c>
       <c r="F61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G61" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 초장거리(220px)에서 22의 관통 화살을 빠르게 사격합니다.</t>
+          <t>초승달 검기로 9 암흑 피해를 입히고 체력 4를 흡혈합니다.</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/arrow_시/arrow_1_32px_pastel.png</t>
+          <t>res://assets/06_회복_치유/moon_light_월/moon_light_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>검술</t>
+          <t>무</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>검술 (무기/연타)</t>
+          <t>무 (무/대포탄)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>weapon</t>
+          <t>heal</t>
         </is>
       </c>
       <c r="F62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G62" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 26의 예리한 검기로 적을 빠르게 2회 연속 베어 넘깁니다.</t>
+          <t>거대한 무 대포탄을 발사하여 착탄 지점에 15의 묵직한 폭발 물리 피해를 입힙니다.</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/sword_검/sword_1_32px_pastel.png</t>
+          <t>res://assets/05_회복_치유/radish_무/radish_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>방패</t>
+          <t>마</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>방패 (방어/버프)</t>
+          <t>마 (산약/마비침)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>defense</t>
+          <t>heal</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G63" t="n">
         <v>12</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 방어 결계를 펼쳐 주변 모든 아군 타워의 공격속도를 +30% 증폭시킵니다.</t>
+          <t>적의 급소에 마비 침을 발사하여 12 피해를 입히고 1초간 이동을 정지(마비)시킵니다.</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>res://assets/02_방어_보호/shield_방/shield_1_32px_pastel.png</t>
+          <t>res://assets/05_회복_치유/yam_마/yam_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>성벽</t>
+          <t>묵</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>성벽 (방어/요새)</t>
+          <t>묵 (도토리묵/슬로우)</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>defense</t>
+          <t>heal</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G64" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 사거리 내 진입한 적들의 이동속도를 50% 영구 감속시킵니다.</t>
+          <t>끈적끈적한 도토리묵 덩어리를 뿜어내어 10 피해 및 적 이동속도를 60% 대폭 감속시킵니다.</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>res://assets/02_방어_보호/wall_성/wall_1_32px_pastel.png</t>
+          <t>res://assets/05_회복_치유/jelly_묵/jelly_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>벼락</t>
+          <t>북</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>벼락 (원소/감전)</t>
+          <t>북 (전쟁의북/고동)</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>skill</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G65" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 30의 강력한 뇌전을 떨어뜨려 최대 3체의 적에게 연쇄 감전 피해를 입힙니다.</t>
+          <t>둥둥 울리는 북소리로 10 음파 피해를 주며, 주변 아군 타워 공격속도를 +40% 가속합니다.</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/lightning_뇌/lightning_1_32px_pastel.png</t>
+          <t>res://assets/06_버프_유틸/drum_북/drum_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>폭풍</t>
+          <t>기</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>폭풍 (원소/소용돌이)</t>
+          <t>기 (기공/관통기공파)</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>skill</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G66" t="n">
         <v>20</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 거대한 소용돌이를 소환하여 범위 내 적들을 지속적으로 갈아냅니다.</t>
+          <t>일직선상 모든 적을 관통하는 푸른 기공파를 발사하여 20의 강력한 관통 피해를 입힙니다.</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/wind_풍/wind_1_32px_pastel.png</t>
+          <t>res://assets/06_버프_유틸/ki_기/ki_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>바람</t>
+          <t>속</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>바람 (원소/돌풍)</t>
+          <t>속 (속도/고속연사)</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>skill</t>
         </is>
       </c>
       <c r="F67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G67" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 강한 돌풍을 날려 적을 뒤로 넉백시킵니다.</t>
+          <t>공격 쿨타임이 0.25초로 극도로 빨라 초당 4회 이상의 고속 활자 난사를 퍼붓습니다.</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/wind_풍/wind_1_32px_pastel.png</t>
+          <t>res://assets/06_버프_유틸/speed_속/speed_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>치유</t>
+          <t>능</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>치유 (회복/성역)</t>
+          <t>능 (능력/마력증폭)</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>heal</t>
+          <t>skill</t>
         </is>
       </c>
       <c r="F68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G68" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 매 웨이브 클리어 시 플레이어 기지 체력을 +2 추가 회복합니다.</t>
+          <t>적에게 16 마력 광선을 쏘며 마력 표식을 남겨, 대상이 받는 모든 타워 피해를 +30% 증폭시킵니다.</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>res://assets/06_회복_치유/life_sprout_생/life_sprout_1_32px_pastel.png</t>
+          <t>res://assets/06_버프_유틸/mana_능/mana_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>생명</t>
+          <t>세</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>생명 (회복/축복)</t>
+          <t>세 (기세/압도)</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>heal</t>
+          <t>basic</t>
         </is>
       </c>
       <c r="F69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G69" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 기지의 최대 체력을 +5 영구 증가시킵니다.</t>
+          <t>도도한 기세로 8 피해를 입히고 다음 내 카드의 공격력을 +4 증가시킵니다.</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>res://assets/06_회복_치유/life_sprout_생/life_sprout_1_32px_pastel.png</t>
+          <t>res://assets/07_버프_유틸/power_surge_세/power_surge_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>맹독</t>
+          <t>망</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>맹독 (원소/부식)</t>
+          <t>망 (포획망/속박)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2글자</t>
+          <t>1글자</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>2티어 (상위)</t>
+          <t>1티어 (기본)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>skill</t>
         </is>
       </c>
       <c r="F70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G70" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 적에게 초당 8의 치명적인 맹독 부식 피해를 부여합니다.</t>
+          <t>거대한 올가미 그물을 투척하여 14 피해를 입히고 적들을 1.2초간 묶어둡니다(속박).</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/dark_orb_암/dark_orb_1_32px_pastel.png</t>
+          <t>res://assets/06_버프_유틸/net_망/net_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>호랑</t>
+          <t>불꽃</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>호랑 (생물/맹수)</t>
+          <t>불꽃 (원소/폭발)</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3468,35 +3468,35 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>summon</t>
+          <t>element</t>
         </is>
       </c>
       <c r="F71" t="n">
         <v>2</v>
       </c>
       <c r="G71" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 28의 맹수 타격으로 적의 방어도를 무시하고 물어뜯습니다.</t>
+          <t>[2글자 상위 타워] 24의 강력한 광역 화염 폭발을 일으키고 적들을 불태웁니다.</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/bear_곰/bear_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/fire_불/fire_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>마법</t>
+          <t>얼음</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>마법 (마법/비전)</t>
+          <t>얼음 (원소/빙결)</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3518,28 +3518,28 @@
         <v>2</v>
       </c>
       <c r="G72" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 일직선상의 적을 모두 꿰뚫는 관통 비전 탄환을 발사합니다.</t>
+          <t>[2글자 상위 타워] 18의 냉기 피해를 주고 적의 이동속도를 75% 둔화시킵니다.</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/light_holy_광/light_holy_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/ice_빙/ice_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>보물</t>
+          <t>화살</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>보물 (유틸/황금)</t>
+          <t>화살 (무기/원거리)</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3554,35 +3554,35 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>weapon</t>
         </is>
       </c>
       <c r="F73" t="n">
         <v>2</v>
       </c>
       <c r="G73" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 이 타워가 적을 처치하면 2배의 골드를 획득합니다.</t>
+          <t>[2글자 상위 타워] 초장거리(220px)에서 22의 관통 화살을 빠르게 사격합니다.</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>res://assets/07_버프_유틸/gold_coin_금/gold_coin_1_32px_pastel.png</t>
+          <t>res://assets/01_무기_공격/arrow_시/arrow_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>강철</t>
+          <t>검술</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>강철 (방어/단련)</t>
+          <t>검술 (무기/연타)</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3597,18 +3597,18 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>defense</t>
+          <t>weapon</t>
         </is>
       </c>
       <c r="F74" t="n">
         <v>2</v>
       </c>
       <c r="G74" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 단단한 강철 파편을 투척하여 적을 분쇄합니다.</t>
+          <t>[2글자 상위 타워] 26의 예리한 검기로 적을 빠르게 2회 연속 베어 넘깁니다.</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -3620,12 +3620,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>화염</t>
+          <t>방패</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>화염 (원소/업화)</t>
+          <t>방패 (방어/공속오라)</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3640,88 +3640,88 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="F75" t="n">
         <v>2</v>
       </c>
       <c r="G75" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>[2글자 상위 타워] 전방 부채꼴 범위에 27 피해의 지속 화염 방사를 뿜어냅니다.</t>
+          <t>[2글자 상위 타워] 20의 방어 충격파를 발사하며 주변 모든 아군 타워 공격속도를 +30% 증폭시킵니다.</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/fire_불/fire_1_32px_pastel.png</t>
+          <t>res://assets/02_방어_장비/shield_방/shield_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>호랑이</t>
+          <t>성벽</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>호랑이 (생물/신수)</t>
+          <t>성벽 (방어/감속요새)</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>3글자</t>
+          <t>2글자</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>3티어 (신화)</t>
+          <t>2티어 (상위)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>summon</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="F76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G76" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>[3글자 신화 타워] 50의 압도적인 맹수 포효로 적들을 공포에 질리게 하고 전방을 도륙합니다.</t>
+          <t>[2글자 상위 타워] 22의 육중한 요새 방어탄을 발사하며 사거리 내 진입한 적들의 속도를 50% 영구 감속시킵니다.</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/bear_곰/bear_1_32px_pastel.png</t>
+          <t>res://assets/02_방어_장비/castle_성/castle_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>불벼락</t>
+          <t>벼락</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>불벼락 (원소/천벌)</t>
+          <t>벼락 (원소/감전)</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>3글자</t>
+          <t>2글자</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>3티어 (신화)</t>
+          <t>2티어 (상위)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3730,41 +3730,41 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G77" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>[3글자 신화 타워] 60의 화염 낙뢰 폭격으로 화면 내 다수의 적을 일격에 궤멸시킵니다.</t>
+          <t>[2글자 상위 타워] 30의 강력한 뇌전을 떨어뜨려 최대 3체의 적에게 연쇄 감전 피해를 입힙니다.</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/fire_불/fire_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/lightning_뇌/lightning_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>폭풍우</t>
+          <t>폭풍</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>폭풍우 (원소/재앙)</t>
+          <t>폭풍 (원소/소용돌이)</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>3글자</t>
+          <t>2글자</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>3티어 (신화)</t>
+          <t>2티어 (상위)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3773,14 +3773,14 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G78" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>[3글자 신화 타워] 거대한 비바람 태풍을 일으켜 적 전체를 80% 슬로우 상태로 묶어둡니다.</t>
+          <t>[2글자 상위 타워] 거대한 소용돌이를 소환하여 범위 내 적들을 지속적으로 갈아냅니다.</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -3792,151 +3792,151 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>얼음검</t>
+          <t>바람</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>얼음검 (무기/동결)</t>
+          <t>바람 (원소/돌풍)</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>3글자</t>
+          <t>2글자</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>3티어 (신화)</t>
+          <t>2티어 (상위)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>weapon</t>
+          <t>element</t>
         </is>
       </c>
       <c r="F79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G79" t="n">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>[3글자 신화 타워] 42의 절대영도 검기로 적을 베는 즉시 2초간 완전히 얼려 멈춥니다.</t>
+          <t>[2글자 상위 타워] 강한 돌풍을 날려 적을 뒤로 넉백시킵니다.</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/sword_검/sword_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/wind_풍/wind_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>독화살</t>
+          <t>치유</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>독화살 (무기/맹독)</t>
+          <t>치유 (회복/성역포격)</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>3글자</t>
+          <t>2글자</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>3티어 (신화)</t>
+          <t>2티어 (상위)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>weapon</t>
+          <t>heal</t>
         </is>
       </c>
       <c r="F80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G80" t="n">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>[3글자 신화 타워] 38 피해와 함께 초당 15의 치사량 맹독을 주입하는 화살을 난사합니다.</t>
+          <t>[2글자 상위 타워] 20의 성스러운 빛을 폭격하며, 매 웨이브 클리어 시 기지 HP를 +2 추가 회복합니다.</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/arrow_시/arrow_1_32px_pastel.png</t>
+          <t>res://assets/05_회복_치유/spring_샘/spring_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>대검술</t>
+          <t>생명</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>대검술 (무기/오의)</t>
+          <t>생명 (회복/영혼흡수)</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>3글자</t>
+          <t>2글자</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>3티어 (신화)</t>
+          <t>2티어 (상위)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>weapon</t>
+          <t>heal</t>
         </is>
       </c>
       <c r="F81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G81" t="n">
-        <v>55</v>
+        <v>22</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>[3글자 신화 타워] 55의 초대형 참격 검기를 날려 경로 위의 모든 적을 일도양단합니다.</t>
+          <t>[2글자 상위 타워] 22의 강력한 영혼 흡수탄을 쏘아 기지 최대 체력을 +5 영구 증가시킵니다.</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/sword_검/sword_1_32px_pastel.png</t>
+          <t>res://assets/05_회복_치유/life_생/life_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>용의숨</t>
+          <t>맹독</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>용의숨 (원소/신화)</t>
+          <t>맹독 (원소/부식)</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>3글자</t>
+          <t>2글자</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>3티어 (신화)</t>
+          <t>2티어 (상위)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -3945,105 +3945,621 @@
         </is>
       </c>
       <c r="F82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G82" t="n">
-        <v>70</v>
+        <v>16</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>[3글자 신화 타워] 70의 신화급 드래곤 브레스를 뿜어 전방의 모든 적을 잿더미로 만듭니다.</t>
+          <t>[2글자 상위 타워] 적에게 초당 8의 치명적인 맹독 부식 피해를 부여합니다.</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/dragon_용/dragon_1_32px_pastel.png</t>
+          <t>res://assets/03_원소_마법/dark_orb_암/dark_orb_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>생명수</t>
+          <t>호랑</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>생명수 (회복/기적)</t>
+          <t>호랑 (생물/맹수)</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>3글자</t>
+          <t>2글자</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>3티어 (신화)</t>
+          <t>2티어 (상위)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>heal</t>
+          <t>summon</t>
         </is>
       </c>
       <c r="F83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G83" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>[3글자 신화 타워] 기지 체력을 즉시 +5 회복하고, 전 필드 아군 타워 공속을 +50% 버프합니다.</t>
+          <t>[2글자 상위 타워] 28의 맹수 타격으로 적의 방어도를 무시하고 물어뜯습니다.</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>res://assets/06_회복_치유/life_sprout_생/life_sprout_1_32px_pastel.png</t>
+          <t>res://assets/04_생물_소환/bear_곰/bear_1_32px_pastel.png</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
+          <t>마법</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>마법 (마법/비전)</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>2글자</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>2티어 (상위)</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>2</v>
+      </c>
+      <c r="G84" t="n">
+        <v>25</v>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>[2글자 상위 타워] 일직선상의 적을 모두 꿰뚫는 관통 비전 탄환을 발사합니다.</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>res://assets/03_원소_마법/light_holy_광/light_holy_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>보물</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>보물 (유틸/황금포격)</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>2글자</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>2티어 (상위)</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>skill</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>2</v>
+      </c>
+      <c r="G85" t="n">
+        <v>18</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>[2글자 상위 타워] 18의 눈부신 황금 코인 탄환을 발사하며 적 처치 시 2배의 골드를 획득합니다.</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>res://assets/06_버프_유틸/mana_능/mana_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>강철</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>강철 (방어/강철포)</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>2글자</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>2티어 (상위)</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>defense</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>2</v>
+      </c>
+      <c r="G86" t="n">
+        <v>26</v>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>[2글자 상위 타워] 26의 단단한 강철 볼트를 발사하여 일직선상의 적들을 분쇄합니다.</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>res://assets/02_방어_장비/armor_갑/armor_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>화염</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>화염 (원소/업화)</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>2글자</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>2티어 (상위)</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>2</v>
+      </c>
+      <c r="G87" t="n">
+        <v>27</v>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>[2글자 상위 타워] 전방 부채꼴 범위에 27 피해의 지속 화염 방사를 뿜어냅니다.</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>res://assets/03_원소_마법/fire_불/fire_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>호랑이</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>호랑이 (생물/신수)</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>3글자</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>3티어 (신화)</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>summon</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>3</v>
+      </c>
+      <c r="G88" t="n">
+        <v>50</v>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>[3글자 신화 타워] 50의 압도적인 맹수 포효로 적들을 공포에 질리게 하고 전방을 도륙합니다.</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>res://assets/04_생물_소환/bear_곰/bear_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>불벼락</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>불벼락 (원소/천벌)</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>3글자</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>3티어 (신화)</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>3</v>
+      </c>
+      <c r="G89" t="n">
+        <v>60</v>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>[3글자 신화 타워] 60의 화염 낙뢰 폭격으로 화면 내 다수의 적을 일격에 궤멸시킵니다.</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>res://assets/03_원소_마법/fire_불/fire_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>폭풍우</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>폭풍우 (원소/재앙)</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>3글자</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>3티어 (신화)</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>3</v>
+      </c>
+      <c r="G90" t="n">
+        <v>45</v>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>[3글자 신화 타워] 거대한 비바람 태풍을 일으켜 적 전체를 80% 슬로우 상태로 묶어둡니다.</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>res://assets/03_원소_마법/wind_풍/wind_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>얼음검</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>얼음검 (무기/동결)</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>3글자</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>3티어 (신화)</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>3</v>
+      </c>
+      <c r="G91" t="n">
+        <v>42</v>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>[3글자 신화 타워] 42의 절대영도 검기로 적을 베는 즉시 2초간 완전히 얼려 멈춥니다.</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>res://assets/01_무기_공격/sword_검/sword_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>독화살</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>독화살 (무기/맹독)</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>3글자</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>3티어 (신화)</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>3</v>
+      </c>
+      <c r="G92" t="n">
+        <v>38</v>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>[3글자 신화 타워] 38 피해와 함께 초당 15의 치사량 맹독을 주입하는 화살을 난사합니다.</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>res://assets/01_무기_공격/arrow_시/arrow_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>대검술</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>대검술 (무기/오의)</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>3글자</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>3티어 (신화)</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>3</v>
+      </c>
+      <c r="G93" t="n">
+        <v>55</v>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>[3글자 신화 타워] 55의 초대형 참격 검기를 날려 경로 위의 모든 적을 일도양단합니다.</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>res://assets/01_무기_공격/sword_검/sword_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>용의숨</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>용의숨 (원소/신화)</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>3글자</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>3티어 (신화)</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>3</v>
+      </c>
+      <c r="G94" t="n">
+        <v>70</v>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>[3글자 신화 타워] 70의 신화급 드래곤 브레스를 뿜어 전방의 모든 적을 잿더미로 만듭니다.</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>res://assets/04_생물_소환/dragon_용/dragon_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>생명수</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>생명수 (회복/기적폭격)</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>3글자</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>3티어 (신화)</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>heal</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>3</v>
+      </c>
+      <c r="G95" t="n">
+        <v>45</v>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>[3글자 신화 타워] 45의 성스러운 기적 폭격을 쏟아부으며 기지 체력 +5 회복 및 전 필드 아군 타워 공속을 +50% 버프합니다.</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>res://assets/05_회복_치유/spring_샘/spring_1_32px_pastel.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
           <t>철옹성</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>철옹성 (방어/무적)</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>철옹성 (방어/요새포)</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
         <is>
           <t>3글자</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr">
+      <c r="D96" t="inlineStr">
         <is>
           <t>3티어 (신화)</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
+      <c r="E96" t="inlineStr">
         <is>
           <t>defense</t>
         </is>
       </c>
-      <c r="F84" t="n">
+      <c r="F96" t="n">
         <v>3</v>
       </c>
-      <c r="G84" t="n">
-        <v>30</v>
-      </c>
-      <c r="H84" t="inlineStr">
-        <is>
-          <t>[3글자 신화 타워] 절대적인 방어 요새를 구축하여 기지에 가해지는 피해를 대폭 흡수합니다.</t>
-        </is>
-      </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>res://assets/02_방어_보호/wall_성/wall_1_32px_pastel.png</t>
+      <c r="G96" t="n">
+        <v>48</v>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>[3글자 신화 타워] 48의 무적 요새포 3연사를 발사하여 다가오는 모든 적들을 산산조각 내고 멀리 밀어냅니다.</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>res://assets/02_방어_장비/castle_성/castle_1_32px_pastel.png</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(balance): Assign ㄱ, ㅡ, ㅜ as RARE high-value tiles with reduced weighted draw rate (1/5) and golden visual styling
</commit_message>
<xml_diff>
--- a/word_assets_all.xlsx
+++ b/word_assets_all.xlsx
@@ -507,7 +507,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L312"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58.4" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -19207,7 +19207,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="41.9" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
@@ -19479,7 +19479,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="41.2" customWidth="1" min="1" max="1"/>
     <col width="16.2" customWidth="1" min="2" max="2"/>
@@ -19530,7 +19530,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>초성/종성 자음</t>
+          <t>🌟 희귀 자모 (Rare, 낮은 확률)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -19545,7 +19545,7 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>기본 풀 (상시 획득)</t>
+          <t>희귀 드롭 풀 (가중치 20, 일반의 1/5)</t>
         </is>
       </c>
     </row>
@@ -19989,7 +19989,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>중성 모음</t>
+          <t>🌟 희귀 자모 (Rare, 낮은 확률)</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -20004,7 +20004,7 @@
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>스타팅 덱 &amp; 기본 풀</t>
+          <t>희귀 드롭 풀 (가중치 20, 일반의 1/5)</t>
         </is>
       </c>
     </row>
@@ -20016,7 +20016,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>중성 모음</t>
+          <t>🌟 희귀 자모 (Rare, 낮은 확률)</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -20031,7 +20031,7 @@
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>기본 풀 (상시 획득)</t>
+          <t>희귀 드롭 풀 (가중치 20, 일반의 1/5)</t>
         </is>
       </c>
     </row>

</xml_diff>